<commit_message>
Implementar asignación de alertas a usuarios específicos
</commit_message>
<xml_diff>
--- a/backend/old_data/MAREAS 2025.xlsx
+++ b/backend/old_data/MAREAS 2025.xlsx
@@ -5,18 +5,16 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Gestión de mareas\Administración\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desarrollo\_INIDEP\OBS\Mareas\gestion-mareas-monorepo\backend\old_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC9519CB-0FBD-4BD5-8567-7D7DCF5F92B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B58A08AE-E2FF-4723-A8A3-38B939923789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="4575" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
     <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
-    <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
-    <sheet name="Hoja4" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$V$207</definedName>
@@ -26915,22 +26913,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>